<commit_message>
integracion con muestras API
</commit_message>
<xml_diff>
--- a/Registros Pendientes/RegistroAuxiliar.xlsx
+++ b/Registros Pendientes/RegistroAuxiliar.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,244 +451,79 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2203798</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ERROR</t>
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2298814</v>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2203840</v>
+        <v>2298815</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2203841</v>
+        <v>2298816</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2203842</v>
+        <v>2298817</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2203909</v>
+        <v>2298818</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2203910</v>
+        <v>2298830</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2203911</v>
+        <v>2298831</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2203912</v>
+        <v>2298832</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2203913</v>
+        <v>2298833</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2203914</v>
+        <v>2298834</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2203915</v>
+        <v>2298835</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2203916</v>
+        <v>2298836</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2203917</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>2203918</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>2203920</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>2203921</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>2203922</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>2203923</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>2203924</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>2203925</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>2203926</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>2203927</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>2203928</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>2203929</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>2203930</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>2203931</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>2203932</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>2203933</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>2203934</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>2203935</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>2203936</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>2203937</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>2220091</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>2220092</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>2220093</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>2220094</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>2220095</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>2220096</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>2220097</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>2220098</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>2220099</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>2220100</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>2220101</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>2225271</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>2225272</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>2228150</v>
+        <v>2298837</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A48"/>
+  <autoFilter ref="A1:A15"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix funcional BOG formato fechas
</commit_message>
<xml_diff>
--- a/Registros Pendientes/RegistroAuxiliar.xlsx
+++ b/Registros Pendientes/RegistroAuxiliar.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$A$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,8 +687,23 @@
         <v>2228150</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>2242676</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2242679</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>2242680</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:A48"/>
+  <autoFilter ref="A1:A51"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>